<commit_message>
feat: localize Excel calculator to Russian and prefill demo parameters
</commit_message>
<xml_diff>
--- a/adaptive_lock_ev_calculator.xlsx
+++ b/adaptive_lock_ev_calculator.xlsx
@@ -425,20 +425,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Калькулятор не торгует. Он только рассчитывает следующий допустимый шаг системы.</t>
+          <t>Калькулятор Adaptive Lock EV (демо)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Назначение: расчет следующего допустимого шага системы.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Заполните вручную Broker_Params, Symbol_Params, Current_Positions, Market_Data.</t>
+          <t>Важно: калькулятор не торгует, только рассчитывает.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Все параметры ниже заполнены демо-данными на русском языке.</t>
         </is>
       </c>
     </row>
@@ -453,18 +467,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TriggerDown</t>
-        </is>
-      </c>
-      <c r="B1">
-        <f>Market_Data!B2-Calculations!B12*Symbol_Params!B3</f>
-        <v/>
+          <t>Демо-данные заполнены</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -480,7 +490,15 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Демо-данные заполнены</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -493,7 +511,15 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Демо-данные заполнены</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -506,7 +532,15 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Демо-данные заполнены</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -517,9 +551,207 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Параметр</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Баланс счёта</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Эквити</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Плечо</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1:100</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Спред (пункты)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Комиссия за 1 лот</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Проскальзывание (пункты)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Своп BUY</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Своп SELL</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Маржа на 1 лот</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Мин. лот</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Шаг лота</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Макс. лот</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>100</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -530,9 +762,179 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Параметр</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Символ</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>EURUSD</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Digits</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Точность</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Шаг цены</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tick Size</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Размер тика</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tick Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Стоимость тика</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pip Value 1 Lot</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Стоимость пункта</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Contract Size</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Контракт</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ATR Period Short</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>14</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ATR Period Long</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EMA Period</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>50</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -543,9 +945,192 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Параметр</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Base Lock Buy Lot</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Base Lock Sell Lot</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Q Min</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q Max</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Max Total Lot</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Max Exposure</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Z Entry Level</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>V Mean Revert Max</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>V Volatile Stop</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DD Stress Level</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DD Escape Level</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DD Beta Protection</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Beta Min</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Beta Max</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Beta DD Protection</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Min EV Required</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Safety Cost Multiplier</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -558,7 +1143,15 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Демо-данные заполнены</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -569,9 +1162,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Параметр</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Текущая цена</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.0985</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ATR Short</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.0018</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ATR Long</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.002</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Текущий DD</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Последний PnL 10 циклов</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -582,7 +1248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,58 +1273,69 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>MIN(ABS(B1)/2,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>MIN(MAX(System_Params!B4+System_Params!B4*B3,System_Params!B4),System_Params!B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>IF(Market_Data!B6&gt;System_Params!B13,System_Params!B17,0.7-0.4*B3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>(Broker_Params!B5*B4*Symbol_Params!B7)+(Broker_Params!B6*B4)+(Broker_Params!B7*B4*Symbol_Params!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EV</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>(6*B4*Symbol_Params!B7)-B6</f>
+        <v/>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Q_Final</t>
+          <t>MinMovePoints</t>
         </is>
       </c>
       <c r="B8">
-        <f>0.02</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PipValue</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>TotalCost</t>
-        </is>
-      </c>
-      <c r="B10">
-        <f>1.2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>1.2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>MinMovePoints</t>
-        </is>
-      </c>
-      <c r="B12">
-        <f>(B10*B11)/(B8*B9)</f>
+        <f>(B6*System_Params!B19)/(B4*Symbol_Params!B7)</f>
         <v/>
       </c>
     </row>
@@ -675,7 +1352,15 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Демо-данные заполнены</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -686,18 +1371,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TriggerUp</t>
-        </is>
-      </c>
-      <c r="B1">
-        <f>Market_Data!B2+Calculations!B12*Symbol_Params!B3</f>
-        <v/>
+          <t>Демо-данные заполнены</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add demo open lock positions and updated current price to Excel calculator
</commit_message>
<xml_diff>
--- a/adaptive_lock_ev_calculator.xlsx
+++ b/adaptive_lock_ev_calculator.xlsx
@@ -1141,15 +1141,102 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Демо-данные заполнены</t>
-        </is>
-      </c>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Лот</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Цена открытия</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Плавающий PnL</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Убыток (USD)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Убыток (пункты)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.17385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>минусовой замок</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>-144.06</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.17175</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>противоположная нога</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1184,7 +1271,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.1</v>
+        <v>1.17193</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
fix: make Excel calculator compute next-step recommendations with demo lock data
</commit_message>
<xml_diff>
--- a/adaptive_lock_ev_calculator.xlsx
+++ b/adaptive_lock_ev_calculator.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,10 +449,10 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Все параметры ниже заполнены демо-данными на русском языке.</t>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Логика следующего шага рассчитывается на листах Calculations/Scenario_Up/Scenario_Down/Recommendations.</t>
         </is>
       </c>
     </row>
@@ -467,14 +467,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Демо-данные заполнены</t>
-        </is>
+          <t>TriggerDown</t>
+        </is>
+      </c>
+      <c r="B1">
+        <f>Market_Data!B2-Calculations!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>IF(AND(Calculations!B1&lt;-System_Params!B8,Calculations!B3="MEAN_REVERT",Calculations!B14="YES",Calculations!B15="ALLOW"),"OPEN","NO_ACTION")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>IF(B2="OPEN","BUY","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>IF(B2="OPEN",Calculations!B6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>IF(B2="OPEN","Mean reversion BUY","Блокировка условий")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -945,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1083,51 +1131,41 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Beta Min</t>
+          <t>Beta DD Protection</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Beta Max</t>
+          <t>Min EV Required</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Beta DD Protection</t>
+          <t>Safety Cost Multiplier</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Min EV Required</t>
+          <t>Expected Mu</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Safety Cost Multiplier</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1141,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1185,6 +1223,15 @@
           <t>Убыток (пункты)</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Сумма BUY</t>
+        </is>
+      </c>
+      <c r="K1">
+        <f>SUMIFS(C2:C100,B2:B100,"BUY")</f>
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1201,8 +1248,9 @@
       <c r="D2" t="n">
         <v>1.17385</v>
       </c>
-      <c r="E2" t="n">
-        <v>-10.5</v>
+      <c r="E2">
+        <f>(Market_Data!B2-D2)/Symbol_Params!B4*C2*Symbol_Params!B7</f>
+        <v/>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1213,6 +1261,15 @@
         <v>-144.06</v>
       </c>
       <c r="H2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Сумма SELL</t>
+        </is>
+      </c>
+      <c r="K2">
+        <f>SUMIFS(C2:C100,B2:B100,"SELL")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1229,7 +1286,10 @@
       <c r="D3" t="n">
         <v>1.17175</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3">
+        <f>(D3-Market_Data!B2)/Symbol_Params!B4*C3*Symbol_Params!B7</f>
+        <v/>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>противоположная нога</t>
@@ -1281,7 +1341,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.0985</v>
+        <v>1.1726</v>
       </c>
     </row>
     <row r="4">
@@ -1301,7 +1361,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.002</v>
+        <v>0.0024</v>
       </c>
     </row>
     <row r="6">
@@ -1335,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1363,66 +1423,143 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Regime</t>
         </is>
       </c>
       <c r="B3">
-        <f>MIN(ABS(B1)/2,1)</f>
+        <f>IF(B2&gt;System_Params!B10,"VOLATILE",IF(B2&lt;System_Params!B9,"MEAN_REVERT","NEUTRAL"))</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="B4">
-        <f>MIN(MAX(System_Params!B4+System_Params!B4*B3,System_Params!B4),System_Params!B5)</f>
+        <f>MIN(ABS(B1)/2,1)</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="B5">
-        <f>IF(Market_Data!B6&gt;System_Params!B13,System_Params!B17,0.7-0.4*B3)</f>
+        <f>MIN(MAX(System_Params!B4+System_Params!B4*B4,System_Params!B4),System_Params!B5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Q adj</t>
         </is>
       </c>
       <c r="B6">
-        <f>(Broker_Params!B5*B4*Symbol_Params!B7)+(Broker_Params!B6*B4)+(Broker_Params!B7*B4*Symbol_Params!B7)</f>
+        <f>IF(B3="NEUTRAL",B5*0.5,IF(B3="VOLATILE",0,B5))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EV</t>
+          <t>Beta</t>
         </is>
       </c>
       <c r="B7">
-        <f>(6*B4*Symbol_Params!B7)-B6</f>
+        <f>IF(Market_Data!B6&gt;System_Params!B13,System_Params!B14,0.7-0.4*B4)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>(Broker_Params!B5*B6*Symbol_Params!B7)+(Broker_Params!B6*B6)+(Broker_Params!B7*B6*Symbol_Params!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EV</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>(System_Params!B17*B6*Symbol_Params!B7)-B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>MinMovePoints</t>
         </is>
       </c>
-      <c r="B8">
-        <f>(B6*System_Params!B19)/(B4*Symbol_Params!B7)</f>
+      <c r="B10">
+        <f>(B8*System_Params!B16)/(B6*Symbol_Params!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MinMovePrice</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>B10*Symbol_Params!B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TotalLot</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>Current_Positions!K1+Current_Positions!K2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Exposure</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>ABS(Current_Positions!K1-Current_Positions!K2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RiskOK</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>IF(AND(B12&lt;=System_Params!B6,B13&lt;=System_Params!B7),"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EV_OK</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>IF(B9&gt;System_Params!B15,"ALLOW","BLOCK")</f>
         <v/>
       </c>
     </row>
@@ -1437,14 +1574,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Демо-данные заполнены</t>
-        </is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>Scenario_Up!B2</f>
+        <v/>
+      </c>
+      <c r="C2">
+        <f>Scenario_Up!B3</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>Scenario_Up!B1</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>Scenario_Up!B4</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>Scenario_Up!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>Scenario_Down!B2</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>Scenario_Down!B3</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>Scenario_Down!B1</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>Scenario_Down!B4</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>Scenario_Down!B5</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1458,14 +1674,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Демо-данные заполнены</t>
-        </is>
+          <t>TriggerUp</t>
+        </is>
+      </c>
+      <c r="B1">
+        <f>Market_Data!B2+Calculations!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>IF(AND(Calculations!B1&gt;System_Params!B8,Calculations!B3="MEAN_REVERT",Calculations!B14="YES",Calculations!B15="ALLOW"),"OPEN","NO_ACTION")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>IF(B2="OPEN","SELL","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>IF(B2="OPEN",Calculations!B6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>IF(B2="OPEN","Mean reversion SELL","Блокировка условий")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>